<commit_message>
Output files with records for memory and speed up assessment
</commit_message>
<xml_diff>
--- a/Simulations/Parametros.xlsx
+++ b/Simulations/Parametros.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29530"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\julia\Documents\GitHub\normScore\Simulations\CESGA\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\julia\Documents\GitHub\normScore\Simulations\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B4A7DFFB-CFE5-4A69-AEB5-9BD609D0A9EF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6323A2DD-895D-455D-B58A-20B8A5C66192}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="17775" yWindow="5670" windowWidth="21930" windowHeight="12975" xr2:uid="{B7C000AD-72BA-48D6-8B28-D6AA0A1B8253}"/>
+    <workbookView xWindow="18705" yWindow="690" windowWidth="31995" windowHeight="19920" xr2:uid="{B7C000AD-72BA-48D6-8B28-D6AA0A1B8253}"/>
   </bookViews>
   <sheets>
     <sheet name="Pruebas_Item2" sheetId="1" r:id="rId1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="66" uniqueCount="16">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="85" uniqueCount="35">
   <si>
     <t>Combinatiosn from grid</t>
   </si>
@@ -73,6 +73,63 @@
   </si>
   <si>
     <t>Time (min)</t>
+  </si>
+  <si>
+    <t>File</t>
+  </si>
+  <si>
+    <t>output_item2_1000p_n1.log</t>
+  </si>
+  <si>
+    <t>output_item2_5000p_n8.log</t>
+  </si>
+  <si>
+    <t>output_item2_10000p_n1.log</t>
+  </si>
+  <si>
+    <t>output_item2_n1.log</t>
+  </si>
+  <si>
+    <t>output_item2_n2.log</t>
+  </si>
+  <si>
+    <t>output_item2_n2_nt8.log</t>
+  </si>
+  <si>
+    <t>output_item2_n2_nt12.log</t>
+  </si>
+  <si>
+    <t>output_item2_n4.log</t>
+  </si>
+  <si>
+    <t>output_item2_n4_nt4.log</t>
+  </si>
+  <si>
+    <t>output_item2_n4_nt6.log</t>
+  </si>
+  <si>
+    <t>output_item2_n8.log</t>
+  </si>
+  <si>
+    <t>output_item2_n8_nt2.log</t>
+  </si>
+  <si>
+    <t>output_item2_n8_nt3.log</t>
+  </si>
+  <si>
+    <t>output_item2_n16.log</t>
+  </si>
+  <si>
+    <t>output_item2_n24.log</t>
+  </si>
+  <si>
+    <t>output_item2_n32.log</t>
+  </si>
+  <si>
+    <t>output_item2_n48.log</t>
+  </si>
+  <si>
+    <t>output_item2_n64.log</t>
   </si>
 </sst>
 </file>
@@ -424,108 +481,109 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E7120769-FE5F-480F-A628-B613EF527604}">
-  <dimension ref="A1:M21"/>
+  <dimension ref="B1:O21"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="2" max="2" width="21.140625" customWidth="1"/>
-    <col min="3" max="3" width="12.85546875" bestFit="1" customWidth="1"/>
-    <col min="5" max="6" width="7.7109375" customWidth="1"/>
-    <col min="7" max="7" width="12.28515625" customWidth="1"/>
-    <col min="8" max="8" width="5.42578125" customWidth="1"/>
-    <col min="9" max="9" width="19.42578125" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="13.85546875" customWidth="1"/>
-    <col min="11" max="11" width="6.85546875" customWidth="1"/>
+    <col min="3" max="3" width="26.28515625" customWidth="1"/>
+    <col min="4" max="4" width="12.85546875" bestFit="1" customWidth="1"/>
+    <col min="6" max="7" width="7.7109375" customWidth="1"/>
+    <col min="8" max="8" width="12.28515625" customWidth="1"/>
+    <col min="9" max="9" width="5.42578125" customWidth="1"/>
+    <col min="10" max="10" width="19.42578125" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="13.85546875" customWidth="1"/>
+    <col min="12" max="12" width="6.85546875" customWidth="1"/>
+    <col min="15" max="15" width="26" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A1" t="s">
+    <row r="1" spans="2:15" x14ac:dyDescent="0.25">
+      <c r="B1" t="s">
         <v>3</v>
       </c>
-      <c r="B1" t="s">
+      <c r="C1" t="s">
         <v>0</v>
       </c>
-      <c r="C1" t="s">
-        <v>1</v>
-      </c>
       <c r="D1" t="s">
+        <v>1</v>
+      </c>
+      <c r="E1" t="s">
         <v>2</v>
       </c>
-      <c r="E1" t="s">
+      <c r="F1" t="s">
         <v>11</v>
       </c>
-      <c r="F1" t="s">
+      <c r="G1" t="s">
         <v>12</v>
       </c>
-      <c r="G1" t="s">
+      <c r="H1" t="s">
         <v>13</v>
       </c>
-      <c r="H1" t="s">
+      <c r="I1" t="s">
         <v>9</v>
       </c>
-      <c r="I1" t="s">
+      <c r="J1" t="s">
         <v>5</v>
       </c>
-      <c r="J1" t="s">
+      <c r="K1" t="s">
         <v>6</v>
       </c>
-      <c r="K1" t="s">
+      <c r="L1" t="s">
         <v>10</v>
       </c>
-      <c r="L1" t="s">
+      <c r="M1" t="s">
         <v>14</v>
       </c>
-      <c r="M1" t="s">
+      <c r="N1" t="s">
         <v>15</v>
       </c>
-    </row>
-    <row r="2" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A2">
+      <c r="O1" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="2" spans="2:15" x14ac:dyDescent="0.25">
+      <c r="B2">
         <v>100</v>
       </c>
-      <c r="B2">
+      <c r="C2">
         <v>360</v>
       </c>
-      <c r="C2">
-        <f>B2*9</f>
+      <c r="D2">
+        <f>C2*9</f>
         <v>3240</v>
       </c>
-      <c r="D2">
+      <c r="E2">
         <v>2</v>
       </c>
-      <c r="E2">
-        <v>1</v>
-      </c>
       <c r="F2">
         <v>1</v>
       </c>
       <c r="G2">
+        <v>1</v>
+      </c>
+      <c r="H2">
         <v>2</v>
       </c>
-      <c r="H2" t="s">
-        <v>7</v>
-      </c>
-      <c r="L2">
+      <c r="I2" t="s">
+        <v>7</v>
+      </c>
+      <c r="M2">
         <v>46</v>
       </c>
-      <c r="M2">
-        <f>L2/60</f>
+      <c r="N2">
+        <f>M2/60</f>
         <v>0.76666666666666672</v>
       </c>
     </row>
-    <row r="3" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A3">
+    <row r="3" spans="2:15" x14ac:dyDescent="0.25">
+      <c r="B3">
         <v>1000</v>
       </c>
-      <c r="B3">
+      <c r="C3">
         <v>359</v>
       </c>
-      <c r="C3">
-        <f>B3*9</f>
+      <c r="D3">
+        <f>C3*9</f>
         <v>3231</v>
       </c>
-      <c r="D3">
-        <v>1</v>
-      </c>
       <c r="E3">
         <v>1</v>
       </c>
@@ -535,42 +593,45 @@
       <c r="G3">
         <v>1</v>
       </c>
-      <c r="H3" t="s">
-        <v>7</v>
-      </c>
-      <c r="I3">
+      <c r="H3">
+        <v>1</v>
+      </c>
+      <c r="I3" t="s">
+        <v>7</v>
+      </c>
+      <c r="J3">
         <v>18.82</v>
       </c>
-      <c r="J3">
+      <c r="K3">
         <v>192.67</v>
       </c>
-      <c r="K3" t="s">
+      <c r="L3" t="s">
         <v>8</v>
       </c>
-      <c r="L3">
+      <c r="M3">
         <f>4*60+5</f>
         <v>245</v>
       </c>
-      <c r="M3">
-        <f t="shared" ref="M3:M21" si="0">L3/60</f>
+      <c r="N3">
+        <f t="shared" ref="N3:N21" si="0">M3/60</f>
         <v>4.083333333333333</v>
       </c>
-    </row>
-    <row r="4" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A4">
+      <c r="O3" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="4" spans="2:15" x14ac:dyDescent="0.25">
+      <c r="B4">
         <v>5000</v>
       </c>
-      <c r="B4">
+      <c r="C4">
         <f>360</f>
         <v>360</v>
       </c>
-      <c r="C4">
-        <f>B4*9</f>
+      <c r="D4">
+        <f>C4*9</f>
         <v>3240</v>
       </c>
-      <c r="D4">
-        <v>1</v>
-      </c>
       <c r="E4">
         <v>1</v>
       </c>
@@ -580,76 +641,79 @@
       <c r="G4">
         <v>1</v>
       </c>
-      <c r="H4" t="s">
-        <v>7</v>
-      </c>
-      <c r="L4">
+      <c r="H4">
+        <v>1</v>
+      </c>
+      <c r="I4" t="s">
+        <v>7</v>
+      </c>
+      <c r="M4">
         <f>17*60+17</f>
         <v>1037</v>
       </c>
-      <c r="M4">
+      <c r="N4">
         <f t="shared" si="0"/>
         <v>17.283333333333335</v>
       </c>
     </row>
-    <row r="5" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A5">
+    <row r="5" spans="2:15" x14ac:dyDescent="0.25">
+      <c r="B5">
         <v>5000</v>
       </c>
-      <c r="B5">
+      <c r="C5">
         <v>360</v>
       </c>
-      <c r="C5">
+      <c r="D5">
         <v>3240</v>
       </c>
-      <c r="D5">
+      <c r="E5">
         <v>8</v>
       </c>
-      <c r="E5">
-        <v>1</v>
-      </c>
       <c r="F5">
         <v>1</v>
       </c>
       <c r="G5">
+        <v>1</v>
+      </c>
+      <c r="H5">
         <f>4</f>
         <v>4</v>
       </c>
-      <c r="H5" t="s">
-        <v>7</v>
-      </c>
-      <c r="I5">
+      <c r="I5" t="s">
+        <v>7</v>
+      </c>
+      <c r="J5">
         <v>44.51</v>
       </c>
-      <c r="J5">
+      <c r="K5">
         <v>1.78</v>
       </c>
-      <c r="K5" t="s">
-        <v>7</v>
-      </c>
-      <c r="L5">
+      <c r="L5" t="s">
+        <v>7</v>
+      </c>
+      <c r="M5">
         <f>7*60+7</f>
         <v>427</v>
       </c>
-      <c r="M5">
+      <c r="N5">
         <f t="shared" si="0"/>
         <v>7.1166666666666663</v>
       </c>
-    </row>
-    <row r="6" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A6">
+      <c r="O5" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="6" spans="2:15" x14ac:dyDescent="0.25">
+      <c r="B6">
         <v>10000</v>
       </c>
-      <c r="B6">
+      <c r="C6">
         <v>360</v>
       </c>
-      <c r="C6">
-        <f t="shared" ref="C6:C12" si="1">B6*9</f>
+      <c r="D6">
+        <f t="shared" ref="D6:D12" si="1">C6*9</f>
         <v>3240</v>
       </c>
-      <c r="D6">
-        <v>1</v>
-      </c>
       <c r="E6">
         <v>1</v>
       </c>
@@ -659,41 +723,44 @@
       <c r="G6">
         <v>1</v>
       </c>
-      <c r="H6" t="s">
-        <v>7</v>
-      </c>
-      <c r="I6">
+      <c r="H6">
+        <v>1</v>
+      </c>
+      <c r="I6" t="s">
+        <v>7</v>
+      </c>
+      <c r="J6">
         <v>56.2</v>
       </c>
-      <c r="J6">
+      <c r="K6">
         <v>575.47</v>
       </c>
-      <c r="K6" t="s">
+      <c r="L6" t="s">
         <v>8</v>
       </c>
-      <c r="L6">
+      <c r="M6">
         <f>33*60+20</f>
         <v>2000</v>
       </c>
-      <c r="M6">
+      <c r="N6">
         <f t="shared" si="0"/>
         <v>33.333333333333336</v>
       </c>
-    </row>
-    <row r="7" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A7" t="s">
-        <v>4</v>
-      </c>
-      <c r="B7">
+      <c r="O6" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="7" spans="2:15" x14ac:dyDescent="0.25">
+      <c r="B7" t="s">
+        <v>4</v>
+      </c>
+      <c r="C7">
         <v>1440</v>
       </c>
-      <c r="C7">
+      <c r="D7">
         <f t="shared" si="1"/>
         <v>12960</v>
       </c>
-      <c r="D7">
-        <v>1</v>
-      </c>
       <c r="E7">
         <v>1</v>
       </c>
@@ -701,643 +768,691 @@
         <v>1</v>
       </c>
       <c r="G7">
+        <v>1</v>
+      </c>
+      <c r="H7">
         <v>700</v>
       </c>
-      <c r="H7" t="s">
+      <c r="I7" t="s">
         <v>8</v>
       </c>
-      <c r="I7">
+      <c r="J7">
         <v>83.43</v>
       </c>
-      <c r="J7">
+      <c r="K7">
         <v>584.33000000000004</v>
       </c>
-      <c r="K7" t="s">
+      <c r="L7" t="s">
         <v>8</v>
       </c>
-      <c r="L7">
+      <c r="M7">
         <f>56*60+43</f>
         <v>3403</v>
       </c>
-      <c r="M7">
+      <c r="N7">
         <f t="shared" si="0"/>
         <v>56.716666666666669</v>
       </c>
-    </row>
-    <row r="8" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A8" t="s">
-        <v>4</v>
-      </c>
-      <c r="B8">
+      <c r="O7" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="8" spans="2:15" x14ac:dyDescent="0.25">
+      <c r="B8" t="s">
+        <v>4</v>
+      </c>
+      <c r="C8">
         <v>1440</v>
       </c>
-      <c r="C8">
+      <c r="D8">
         <f t="shared" si="1"/>
         <v>12960</v>
       </c>
-      <c r="D8">
+      <c r="E8">
         <v>2</v>
       </c>
-      <c r="E8">
-        <v>1</v>
-      </c>
       <c r="F8">
         <v>1</v>
       </c>
       <c r="G8">
+        <v>1</v>
+      </c>
+      <c r="H8">
         <v>1.37</v>
       </c>
-      <c r="H8" t="s">
-        <v>7</v>
-      </c>
-      <c r="I8">
+      <c r="I8" t="s">
+        <v>7</v>
+      </c>
+      <c r="J8">
         <v>59.02</v>
       </c>
-      <c r="J8">
+      <c r="K8">
         <v>826.26</v>
       </c>
-      <c r="K8" t="s">
+      <c r="L8" t="s">
         <v>8</v>
       </c>
-      <c r="L8">
+      <c r="M8">
         <f>51*60+32</f>
         <v>3092</v>
       </c>
-      <c r="M8">
+      <c r="N8">
         <f t="shared" si="0"/>
         <v>51.533333333333331</v>
       </c>
-    </row>
-    <row r="9" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A9" t="s">
-        <v>4</v>
-      </c>
-      <c r="B9">
+      <c r="O8" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="9" spans="2:15" x14ac:dyDescent="0.25">
+      <c r="B9" t="s">
+        <v>4</v>
+      </c>
+      <c r="C9">
         <v>1440</v>
       </c>
-      <c r="C9">
+      <c r="D9">
         <f t="shared" si="1"/>
         <v>12960</v>
       </c>
-      <c r="D9">
-        <v>4</v>
-      </c>
       <c r="E9">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="F9">
         <v>1</v>
       </c>
       <c r="G9">
+        <v>1</v>
+      </c>
+      <c r="H9">
         <v>2.34</v>
       </c>
-      <c r="H9" t="s">
-        <v>7</v>
-      </c>
-      <c r="I9">
+      <c r="I9" t="s">
+        <v>7</v>
+      </c>
+      <c r="J9">
         <v>55.35</v>
       </c>
-      <c r="J9">
+      <c r="K9">
         <v>1.3</v>
       </c>
-      <c r="K9" t="s">
-        <v>7</v>
-      </c>
-      <c r="L9">
+      <c r="L9" t="s">
+        <v>7</v>
+      </c>
+      <c r="M9">
         <f>38*60+15</f>
         <v>2295</v>
       </c>
-      <c r="M9">
+      <c r="N9">
         <f t="shared" si="0"/>
         <v>38.25</v>
       </c>
-    </row>
-    <row r="10" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A10" t="s">
-        <v>4</v>
-      </c>
-      <c r="B10">
+      <c r="O9" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="10" spans="2:15" x14ac:dyDescent="0.25">
+      <c r="B10" t="s">
+        <v>4</v>
+      </c>
+      <c r="C10">
         <v>1440</v>
       </c>
-      <c r="C10">
+      <c r="D10">
         <f t="shared" si="1"/>
         <v>12960</v>
       </c>
-      <c r="D10">
+      <c r="E10">
         <v>8</v>
       </c>
-      <c r="E10">
-        <v>1</v>
-      </c>
       <c r="F10">
         <v>1</v>
       </c>
       <c r="G10">
+        <v>1</v>
+      </c>
+      <c r="H10">
         <v>3.91</v>
       </c>
-      <c r="H10" t="s">
-        <v>7</v>
-      </c>
-      <c r="I10">
+      <c r="I10" t="s">
+        <v>7</v>
+      </c>
+      <c r="J10">
         <v>51.32</v>
       </c>
-      <c r="J10">
+      <c r="K10">
         <v>2</v>
       </c>
-      <c r="K10" t="s">
-        <v>7</v>
-      </c>
-      <c r="L10">
+      <c r="L10" t="s">
+        <v>7</v>
+      </c>
+      <c r="M10">
         <f>32*60+33</f>
         <v>1953</v>
       </c>
-      <c r="M10">
+      <c r="N10">
         <f t="shared" si="0"/>
         <v>32.549999999999997</v>
       </c>
-    </row>
-    <row r="11" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A11" t="s">
-        <v>4</v>
-      </c>
-      <c r="B11">
+      <c r="O10" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="11" spans="2:15" x14ac:dyDescent="0.25">
+      <c r="B11" t="s">
+        <v>4</v>
+      </c>
+      <c r="C11">
         <v>1440</v>
       </c>
-      <c r="C11">
+      <c r="D11">
         <f t="shared" si="1"/>
         <v>12960</v>
       </c>
-      <c r="D11">
+      <c r="E11">
         <v>16</v>
       </c>
-      <c r="E11">
-        <v>1</v>
-      </c>
       <c r="F11">
         <v>1</v>
       </c>
       <c r="G11">
+        <v>1</v>
+      </c>
+      <c r="H11">
         <v>3.91</v>
       </c>
-      <c r="H11" t="s">
-        <v>7</v>
-      </c>
-      <c r="I11">
+      <c r="I11" t="s">
+        <v>7</v>
+      </c>
+      <c r="J11">
         <v>90.08</v>
       </c>
-      <c r="J11">
+      <c r="K11">
         <v>3.52</v>
       </c>
-      <c r="K11" t="s">
-        <v>7</v>
-      </c>
-      <c r="L11">
+      <c r="L11" t="s">
+        <v>7</v>
+      </c>
+      <c r="M11">
         <f>25*60+56</f>
         <v>1556</v>
       </c>
-      <c r="M11">
+      <c r="N11">
         <f t="shared" si="0"/>
         <v>25.933333333333334</v>
       </c>
-    </row>
-    <row r="12" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A12" t="s">
-        <v>4</v>
-      </c>
-      <c r="B12">
+      <c r="O11" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="12" spans="2:15" x14ac:dyDescent="0.25">
+      <c r="B12" t="s">
+        <v>4</v>
+      </c>
+      <c r="C12">
         <v>1440</v>
       </c>
-      <c r="C12">
+      <c r="D12">
         <f t="shared" si="1"/>
         <v>12960</v>
       </c>
-      <c r="D12">
+      <c r="E12">
         <v>24</v>
       </c>
-      <c r="E12">
-        <v>1</v>
-      </c>
       <c r="F12">
         <v>1</v>
       </c>
       <c r="G12">
+        <v>1</v>
+      </c>
+      <c r="H12">
         <v>7.03</v>
       </c>
-      <c r="H12" t="s">
-        <v>7</v>
-      </c>
-      <c r="I12">
+      <c r="I12" t="s">
+        <v>7</v>
+      </c>
+      <c r="J12">
         <v>73.02</v>
       </c>
-      <c r="J12">
+      <c r="K12">
         <v>5.13</v>
       </c>
-      <c r="K12" t="s">
-        <v>7</v>
-      </c>
-      <c r="L12">
+      <c r="L12" t="s">
+        <v>7</v>
+      </c>
+      <c r="M12">
         <f>19*60+42</f>
         <v>1182</v>
       </c>
-      <c r="M12">
+      <c r="N12">
         <f t="shared" si="0"/>
         <v>19.7</v>
       </c>
-    </row>
-    <row r="13" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A13" t="s">
-        <v>4</v>
-      </c>
-      <c r="B13">
+      <c r="O12" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="13" spans="2:15" x14ac:dyDescent="0.25">
+      <c r="B13" t="s">
+        <v>4</v>
+      </c>
+      <c r="C13">
         <v>1440</v>
       </c>
-      <c r="C13">
-        <f t="shared" ref="C13" si="2">B13*9</f>
+      <c r="D13">
+        <f t="shared" ref="D13" si="2">C13*9</f>
         <v>12960</v>
       </c>
-      <c r="D13">
+      <c r="E13">
         <v>32</v>
       </c>
-      <c r="E13">
-        <v>1</v>
-      </c>
       <c r="F13">
         <v>1</v>
       </c>
       <c r="G13">
+        <v>1</v>
+      </c>
+      <c r="H13">
         <v>7.81</v>
       </c>
-      <c r="H13" t="s">
-        <v>7</v>
-      </c>
-      <c r="I13">
+      <c r="I13" t="s">
+        <v>7</v>
+      </c>
+      <c r="J13">
         <v>84.46</v>
       </c>
-      <c r="J13">
+      <c r="K13">
         <v>6.6</v>
       </c>
-      <c r="K13" t="s">
-        <v>7</v>
-      </c>
-      <c r="L13">
+      <c r="L13" t="s">
+        <v>7</v>
+      </c>
+      <c r="M13">
         <f>13*60+24</f>
         <v>804</v>
       </c>
-      <c r="M13">
-        <f>L13/60</f>
+      <c r="N13">
+        <f>M13/60</f>
         <v>13.4</v>
       </c>
-    </row>
-    <row r="14" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A14" t="s">
-        <v>4</v>
-      </c>
-      <c r="B14">
+      <c r="O13" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="14" spans="2:15" x14ac:dyDescent="0.25">
+      <c r="B14" t="s">
+        <v>4</v>
+      </c>
+      <c r="C14">
         <v>1440</v>
       </c>
-      <c r="C14">
-        <f t="shared" ref="C14:C16" si="3">B14*9</f>
+      <c r="D14">
+        <f t="shared" ref="D14:D16" si="3">C14*9</f>
         <v>12960</v>
       </c>
-      <c r="D14">
+      <c r="E14">
         <v>12</v>
-      </c>
-      <c r="E14">
-        <v>2</v>
       </c>
       <c r="F14">
         <v>2</v>
       </c>
       <c r="G14">
+        <v>2</v>
+      </c>
+      <c r="H14">
         <v>7.03</v>
       </c>
-      <c r="H14" t="s">
-        <v>7</v>
-      </c>
-      <c r="I14">
+      <c r="I14" t="s">
+        <v>7</v>
+      </c>
+      <c r="J14">
         <v>38.299999999999997</v>
       </c>
-      <c r="J14">
+      <c r="K14">
         <v>2.69</v>
       </c>
-      <c r="K14" t="s">
-        <v>7</v>
-      </c>
-      <c r="L14">
+      <c r="L14" t="s">
+        <v>7</v>
+      </c>
+      <c r="M14">
         <f>27*60+30</f>
         <v>1650</v>
       </c>
-      <c r="M14">
+      <c r="N14">
         <f t="shared" si="0"/>
         <v>27.5</v>
       </c>
-    </row>
-    <row r="15" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A15" t="s">
-        <v>4</v>
-      </c>
-      <c r="B15">
+      <c r="O14" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="15" spans="2:15" x14ac:dyDescent="0.25">
+      <c r="B15" t="s">
+        <v>4</v>
+      </c>
+      <c r="C15">
         <v>1440</v>
       </c>
-      <c r="C15">
-        <f t="shared" ref="C15" si="4">B15*9</f>
+      <c r="D15">
+        <f t="shared" ref="D15" si="4">C15*9</f>
         <v>12960</v>
       </c>
-      <c r="D15">
+      <c r="E15">
         <v>16</v>
-      </c>
-      <c r="E15">
-        <v>2</v>
       </c>
       <c r="F15">
         <v>2</v>
       </c>
       <c r="G15">
+        <v>2</v>
+      </c>
+      <c r="H15">
         <v>7.81</v>
       </c>
-      <c r="H15" t="s">
-        <v>7</v>
-      </c>
-      <c r="I15">
+      <c r="I15" t="s">
+        <v>7</v>
+      </c>
+      <c r="J15">
         <v>45.24</v>
       </c>
-      <c r="J15">
+      <c r="K15">
         <v>3.53</v>
       </c>
-      <c r="K15" t="s">
-        <v>7</v>
-      </c>
-      <c r="L15">
+      <c r="L15" t="s">
+        <v>7</v>
+      </c>
+      <c r="M15">
         <f>25*60+43</f>
         <v>1543</v>
       </c>
-      <c r="M15">
-        <f>L15/60</f>
+      <c r="N15">
+        <f>M15/60</f>
         <v>25.716666666666665</v>
       </c>
-    </row>
-    <row r="16" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A16" t="s">
-        <v>4</v>
-      </c>
-      <c r="B16">
+      <c r="O15" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="16" spans="2:15" x14ac:dyDescent="0.25">
+      <c r="B16" t="s">
+        <v>4</v>
+      </c>
+      <c r="C16">
         <v>1440</v>
       </c>
-      <c r="C16">
+      <c r="D16">
         <f t="shared" si="3"/>
         <v>12960</v>
       </c>
-      <c r="D16">
+      <c r="E16">
         <v>2</v>
       </c>
-      <c r="E16">
+      <c r="F16">
         <v>8</v>
       </c>
-      <c r="F16">
-        <v>1</v>
-      </c>
       <c r="G16">
+        <v>1</v>
+      </c>
+      <c r="H16">
         <v>4.6900000000000004</v>
       </c>
-      <c r="H16" t="s">
-        <v>7</v>
-      </c>
-      <c r="I16">
+      <c r="I16" t="s">
+        <v>7</v>
+      </c>
+      <c r="J16">
         <v>17.190000000000001</v>
       </c>
-      <c r="J16">
+      <c r="K16">
         <v>825.22</v>
       </c>
-      <c r="K16" t="s">
+      <c r="L16" t="s">
         <v>8</v>
       </c>
-      <c r="L16">
+      <c r="M16">
         <f>52*60+6</f>
         <v>3126</v>
       </c>
-      <c r="M16">
+      <c r="N16">
         <f t="shared" si="0"/>
         <v>52.1</v>
       </c>
-    </row>
-    <row r="17" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A17" t="s">
-        <v>4</v>
-      </c>
-      <c r="B17">
+      <c r="O16" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="17" spans="2:15" x14ac:dyDescent="0.25">
+      <c r="B17" t="s">
+        <v>4</v>
+      </c>
+      <c r="C17">
         <v>1440</v>
       </c>
-      <c r="C17">
-        <f>B17*9</f>
+      <c r="D17">
+        <f>C17*9</f>
         <v>12960</v>
       </c>
-      <c r="D17">
-        <v>4</v>
-      </c>
       <c r="E17">
         <v>4</v>
       </c>
       <c r="F17">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="G17">
+        <v>1</v>
+      </c>
+      <c r="H17">
         <v>3.34</v>
       </c>
-      <c r="H17" t="s">
-        <v>7</v>
-      </c>
-      <c r="I17">
+      <c r="I17" t="s">
+        <v>7</v>
+      </c>
+      <c r="J17">
         <v>56.94</v>
       </c>
-      <c r="J17">
+      <c r="K17">
         <v>1.33</v>
       </c>
-      <c r="K17" t="s">
-        <v>7</v>
-      </c>
-      <c r="L17">
+      <c r="L17" t="s">
+        <v>7</v>
+      </c>
+      <c r="M17">
         <f>33*60+43</f>
         <v>2023</v>
       </c>
-      <c r="M17">
+      <c r="N17">
         <f t="shared" si="0"/>
         <v>33.716666666666669</v>
       </c>
-    </row>
-    <row r="18" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A18" t="s">
-        <v>4</v>
-      </c>
-      <c r="B18">
+      <c r="O17" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="18" spans="2:15" x14ac:dyDescent="0.25">
+      <c r="B18" t="s">
+        <v>4</v>
+      </c>
+      <c r="C18">
         <v>1440</v>
       </c>
-      <c r="C18">
-        <f t="shared" ref="C18:C19" si="5">B18*9</f>
+      <c r="D18">
+        <f t="shared" ref="D18:D19" si="5">C18*9</f>
         <v>12960</v>
       </c>
-      <c r="D18">
+      <c r="E18">
         <v>8</v>
       </c>
-      <c r="E18">
+      <c r="F18">
         <v>2</v>
       </c>
-      <c r="F18">
-        <v>1</v>
-      </c>
       <c r="G18">
+        <v>1</v>
+      </c>
+      <c r="H18">
         <v>4.6900000000000004</v>
       </c>
-      <c r="H18" t="s">
-        <v>7</v>
-      </c>
-      <c r="I18">
+      <c r="I18" t="s">
+        <v>7</v>
+      </c>
+      <c r="J18">
         <v>42.28</v>
       </c>
-      <c r="J18">
+      <c r="K18">
         <v>1.98</v>
       </c>
-      <c r="K18" t="s">
-        <v>7</v>
-      </c>
-      <c r="L18">
+      <c r="L18" t="s">
+        <v>7</v>
+      </c>
+      <c r="M18">
         <f>27*60+26</f>
         <v>1646</v>
       </c>
-      <c r="M18">
+      <c r="N18">
         <f t="shared" si="0"/>
         <v>27.433333333333334</v>
       </c>
-    </row>
-    <row r="19" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A19" t="s">
-        <v>4</v>
-      </c>
-      <c r="B19">
+      <c r="O18" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="19" spans="2:15" x14ac:dyDescent="0.25">
+      <c r="B19" t="s">
+        <v>4</v>
+      </c>
+      <c r="C19">
         <v>1440</v>
       </c>
-      <c r="C19">
+      <c r="D19">
         <f t="shared" si="5"/>
         <v>12960</v>
       </c>
-      <c r="D19">
+      <c r="E19">
         <v>2</v>
       </c>
-      <c r="E19">
+      <c r="F19">
         <v>12</v>
       </c>
-      <c r="F19">
-        <v>1</v>
-      </c>
       <c r="G19">
+        <v>1</v>
+      </c>
+      <c r="H19">
         <v>2.34</v>
       </c>
-      <c r="H19" t="s">
-        <v>7</v>
-      </c>
-      <c r="I19">
+      <c r="I19" t="s">
+        <v>7</v>
+      </c>
+      <c r="J19">
         <v>34.14</v>
       </c>
-      <c r="J19">
+      <c r="K19">
         <v>819.43</v>
       </c>
-      <c r="K19" t="s">
+      <c r="L19" t="s">
         <v>8</v>
       </c>
-      <c r="L19">
+      <c r="M19">
         <f>50*60+52</f>
         <v>3052</v>
       </c>
-      <c r="M19">
+      <c r="N19">
         <f t="shared" si="0"/>
         <v>50.866666666666667</v>
       </c>
-    </row>
-    <row r="20" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A20" t="s">
-        <v>4</v>
-      </c>
-      <c r="B20">
+      <c r="O19" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="20" spans="2:15" x14ac:dyDescent="0.25">
+      <c r="B20" t="s">
+        <v>4</v>
+      </c>
+      <c r="C20">
         <v>1440</v>
       </c>
-      <c r="C20">
-        <f>B20*9</f>
+      <c r="D20">
+        <f>C20*9</f>
         <v>12960</v>
       </c>
-      <c r="D20">
-        <v>4</v>
-      </c>
       <c r="E20">
+        <v>4</v>
+      </c>
+      <c r="F20">
         <v>6</v>
       </c>
-      <c r="F20">
-        <v>1</v>
-      </c>
       <c r="G20">
+        <v>1</v>
+      </c>
+      <c r="H20">
         <v>2.34</v>
       </c>
-      <c r="H20" t="s">
-        <v>7</v>
-      </c>
-      <c r="I20">
+      <c r="I20" t="s">
+        <v>7</v>
+      </c>
+      <c r="J20">
         <v>56.3</v>
       </c>
-      <c r="J20">
+      <c r="K20">
         <v>1.32</v>
       </c>
-      <c r="K20" t="s">
-        <v>7</v>
-      </c>
-      <c r="L20">
+      <c r="L20" t="s">
+        <v>7</v>
+      </c>
+      <c r="M20">
         <f>33*60+49</f>
         <v>2029</v>
       </c>
-      <c r="M20">
+      <c r="N20">
         <f t="shared" si="0"/>
         <v>33.81666666666667</v>
       </c>
-    </row>
-    <row r="21" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A21" t="s">
-        <v>4</v>
-      </c>
-      <c r="B21">
+      <c r="O20" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="21" spans="2:15" x14ac:dyDescent="0.25">
+      <c r="B21" t="s">
+        <v>4</v>
+      </c>
+      <c r="C21">
         <v>1440</v>
       </c>
-      <c r="C21">
-        <f t="shared" ref="C21" si="6">B21*9</f>
+      <c r="D21">
+        <f t="shared" ref="D21" si="6">C21*9</f>
         <v>12960</v>
       </c>
-      <c r="D21">
+      <c r="E21">
         <v>8</v>
       </c>
-      <c r="E21">
+      <c r="F21">
         <v>3</v>
       </c>
-      <c r="F21">
-        <v>1</v>
-      </c>
       <c r="G21">
+        <v>1</v>
+      </c>
+      <c r="H21">
         <v>2.34</v>
       </c>
-      <c r="H21" t="s">
-        <v>7</v>
-      </c>
-      <c r="I21">
+      <c r="I21" t="s">
+        <v>7</v>
+      </c>
+      <c r="J21">
         <v>85.29</v>
       </c>
-      <c r="J21">
+      <c r="K21">
         <v>2</v>
       </c>
-      <c r="K21" t="s">
-        <v>7</v>
-      </c>
-      <c r="L21">
+      <c r="L21" t="s">
+        <v>7</v>
+      </c>
+      <c r="M21">
         <f>27*60+18</f>
         <v>1638</v>
       </c>
-      <c r="M21">
+      <c r="N21">
         <f t="shared" si="0"/>
         <v>27.3</v>
+      </c>
+      <c r="O21" t="s">
+        <v>29</v>
       </c>
     </row>
   </sheetData>

</xml_diff>